<commit_message>
feat: Enhance workbook column visibility handling; add tests for consecutive months and single month scenarios
</commit_message>
<xml_diff>
--- a/backend/src/main/resources/templates/PLANTILLA_PLANILLA_PROCESO_CTN.xlsx
+++ b/backend/src/main/resources/templates/PLANTILLA_PLANILLA_PROCESO_CTN.xlsx
@@ -617,7 +617,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -693,6 +693,9 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1403,7 +1406,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:BQ15"/>
+  <dimension ref="A1:BQ16"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="9.285714285714286" customWidth="1"/>
@@ -2338,8 +2341,19 @@
       <c r="BO15" s="10"/>
       <c r="BP15" s="10"/>
     </row>
+    <row r="16" spans="60:68" x14ac:dyDescent="0.25">
+      <c r="BH16" s="26"/>
+      <c r="BI16" s="26"/>
+      <c r="BJ16" s="26"/>
+      <c r="BK16" s="26"/>
+      <c r="BL16" s="26"/>
+      <c r="BM16" s="26"/>
+      <c r="BN16" s="26"/>
+      <c r="BO16" s="26"/>
+      <c r="BP16" s="26"/>
+    </row>
   </sheetData>
-  <mergeCells count="23">
+  <mergeCells count="24">
     <mergeCell ref="A1:AZ1"/>
     <mergeCell ref="A2:AZ2"/>
     <mergeCell ref="A3:AZ3"/>
@@ -2363,6 +2377,7 @@
     <mergeCell ref="BP6:BP7"/>
     <mergeCell ref="BQ6:BQ7"/>
     <mergeCell ref="BH15:BP15"/>
+    <mergeCell ref="BH16:BP16"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>